<commit_message>
Add test results and templates for NewCustomer functionality in gpt-4o-mini
- Created JSON files for score prompts and template practice results for various versions of CreateNewCustomer and NewCustomer.
- Added detailed applicable and results data for methods such as enterAddress, createAddress, getAddressID, and insertCustomer.
- Included a comprehensive scenario file for NewCustomer functionality covering multiple versions.
</commit_message>
<xml_diff>
--- a/tool/src/dashboard_llms/output/groundtruth_scores/gt_score_qm.xlsx
+++ b/tool/src/dashboard_llms/output/groundtruth_scores/gt_score_qm.xlsx
@@ -444,53 +444,85 @@
           <t>Method</t>
         </is>
       </c>
-      <c r="D1" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="E1" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="F1" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="G1" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="I1" s="1" t="n">
-        <v>6</v>
-      </c>
-      <c r="J1" s="1" t="n">
-        <v>7</v>
-      </c>
-      <c r="K1" s="1" t="n">
-        <v>8</v>
-      </c>
-      <c r="L1" s="1" t="n">
-        <v>9</v>
-      </c>
-      <c r="M1" s="1" t="n">
-        <v>10</v>
-      </c>
-      <c r="N1" s="1" t="n">
-        <v>11</v>
-      </c>
-      <c r="O1" s="1" t="n">
-        <v>12</v>
-      </c>
-      <c r="P1" s="1" t="n">
-        <v>13</v>
-      </c>
-      <c r="Q1" s="1" t="n">
-        <v>14</v>
-      </c>
-      <c r="R1" s="1" t="n">
-        <v>15</v>
-      </c>
-      <c r="S1" s="1" t="n">
-        <v>16</v>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
@@ -559,7 +591,7 @@
         <v>0</v>
       </c>
       <c r="T2" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="3">
@@ -623,7 +655,7 @@
         <v>0</v>
       </c>
       <c r="T3" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="4">
@@ -685,7 +717,7 @@
         <v>0</v>
       </c>
       <c r="T4" t="n">
-        <v>1</v>
+        <v>0.005132846524336591</v>
       </c>
     </row>
     <row r="5">
@@ -749,7 +781,7 @@
         <v>0</v>
       </c>
       <c r="T5" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="6">
@@ -813,7 +845,7 @@
         <v>0</v>
       </c>
       <c r="T6" t="n">
-        <v>1</v>
+        <v>0.2918963240121821</v>
       </c>
     </row>
     <row r="7">
@@ -875,7 +907,7 @@
         <v>0</v>
       </c>
       <c r="T7" t="n">
-        <v>1</v>
+        <v>0.3173653891803561</v>
       </c>
     </row>
     <row r="8">
@@ -939,7 +971,7 @@
         <v>0</v>
       </c>
       <c r="T8" t="n">
-        <v>1</v>
+        <v>0.007080884352209908</v>
       </c>
     </row>
     <row r="9">
@@ -1003,7 +1035,7 @@
         <v>0</v>
       </c>
       <c r="T9" t="n">
-        <v>1</v>
+        <v>0.3044851262843078</v>
       </c>
     </row>
     <row r="10">
@@ -1067,7 +1099,7 @@
         <v>0</v>
       </c>
       <c r="T10" t="n">
-        <v>1</v>
+        <v>0.2918963240121821</v>
       </c>
     </row>
     <row r="11">
@@ -1131,7 +1163,7 @@
         <v>0</v>
       </c>
       <c r="T11" t="n">
-        <v>1</v>
+        <v>0.2918963240121821</v>
       </c>
     </row>
     <row r="12">
@@ -1195,7 +1227,7 @@
         <v>0</v>
       </c>
       <c r="T12" t="n">
-        <v>1</v>
+        <v>0.2918963240121821</v>
       </c>
     </row>
     <row r="13">
@@ -1259,7 +1291,7 @@
         <v>0</v>
       </c>
       <c r="T13" t="n">
-        <v>1</v>
+        <v>0.007080884352209908</v>
       </c>
     </row>
     <row r="14">
@@ -1323,7 +1355,7 @@
         <v>0</v>
       </c>
       <c r="T14" t="n">
-        <v>1</v>
+        <v>0.01730972989451714</v>
       </c>
     </row>
     <row r="15">
@@ -1387,7 +1419,7 @@
         <v>0</v>
       </c>
       <c r="T15" t="n">
-        <v>1</v>
+        <v>0.2918963240121821</v>
       </c>
     </row>
     <row r="16">
@@ -1451,7 +1483,7 @@
         <v>0</v>
       </c>
       <c r="T16" t="n">
-        <v>1</v>
+        <v>0.2918963240121821</v>
       </c>
     </row>
     <row r="17">
@@ -1515,7 +1547,7 @@
         <v>0</v>
       </c>
       <c r="T17" t="n">
-        <v>1</v>
+        <v>0.2918963240121821</v>
       </c>
     </row>
     <row r="18">
@@ -1579,7 +1611,7 @@
         <v>0</v>
       </c>
       <c r="T18" t="n">
-        <v>1</v>
+        <v>0.007080884352209908</v>
       </c>
     </row>
     <row r="19">
@@ -1643,7 +1675,7 @@
         <v>0</v>
       </c>
       <c r="T19" t="n">
-        <v>1</v>
+        <v>0.3044851262843078</v>
       </c>
     </row>
     <row r="20">
@@ -1707,7 +1739,7 @@
         <v>0</v>
       </c>
       <c r="T20" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="21">
@@ -1771,7 +1803,7 @@
         <v>0</v>
       </c>
       <c r="T21" t="n">
-        <v>1</v>
+        <v>0.2918963240121821</v>
       </c>
     </row>
     <row r="22">
@@ -1835,7 +1867,7 @@
         <v>0</v>
       </c>
       <c r="T22" t="n">
-        <v>1</v>
+        <v>0.2918963240121821</v>
       </c>
     </row>
     <row r="23">
@@ -1899,7 +1931,7 @@
         <v>0</v>
       </c>
       <c r="T23" t="n">
-        <v>1</v>
+        <v>0.007080884352209908</v>
       </c>
     </row>
     <row r="24">
@@ -1963,7 +1995,7 @@
         <v>0</v>
       </c>
       <c r="T24" t="n">
-        <v>1</v>
+        <v>0.3044851262843078</v>
       </c>
     </row>
     <row r="25">
@@ -2027,7 +2059,7 @@
         <v>0</v>
       </c>
       <c r="T25" t="n">
-        <v>1</v>
+        <v>0.2918963240121821</v>
       </c>
     </row>
     <row r="26">
@@ -2091,7 +2123,7 @@
         <v>0</v>
       </c>
       <c r="T26" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="27">
@@ -2155,7 +2187,7 @@
         <v>0</v>
       </c>
       <c r="T27" t="n">
-        <v>1</v>
+        <v>0.2918963240121821</v>
       </c>
     </row>
     <row r="28">
@@ -2219,7 +2251,7 @@
         <v>0</v>
       </c>
       <c r="T28" t="n">
-        <v>1</v>
+        <v>0.007080884352209908</v>
       </c>
     </row>
     <row r="29">
@@ -2283,7 +2315,7 @@
         <v>0</v>
       </c>
       <c r="T29" t="n">
-        <v>1</v>
+        <v>0.3044851262843078</v>
       </c>
     </row>
     <row r="30">
@@ -2347,7 +2379,7 @@
         <v>0</v>
       </c>
       <c r="T30" t="n">
-        <v>1</v>
+        <v>0.2918963240121821</v>
       </c>
     </row>
     <row r="31">
@@ -2411,7 +2443,7 @@
         <v>0</v>
       </c>
       <c r="T31" t="n">
-        <v>1</v>
+        <v>0.2918963240121821</v>
       </c>
     </row>
     <row r="32">
@@ -2475,7 +2507,7 @@
         <v>0</v>
       </c>
       <c r="T32" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="33">
@@ -2539,7 +2571,7 @@
         <v>0</v>
       </c>
       <c r="T33" t="n">
-        <v>1</v>
+        <v>0.007080884352209908</v>
       </c>
     </row>
     <row r="34">
@@ -2603,7 +2635,7 @@
         <v>0</v>
       </c>
       <c r="T34" t="n">
-        <v>1</v>
+        <v>0.01730972989451714</v>
       </c>
     </row>
     <row r="35">
@@ -2667,7 +2699,7 @@
         <v>0</v>
       </c>
       <c r="T35" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="36">
@@ -2731,7 +2763,7 @@
         <v>0</v>
       </c>
       <c r="T36" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="37">
@@ -2795,7 +2827,7 @@
         <v>0</v>
       </c>
       <c r="T37" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="38">
@@ -2847,7 +2879,7 @@
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
       <c r="T38" t="n">
-        <v>1</v>
+        <v>0.1224486876578283</v>
       </c>
     </row>
     <row r="39">
@@ -2911,7 +2943,7 @@
         <v>0</v>
       </c>
       <c r="T39" t="n">
-        <v>1</v>
+        <v>0.2918963240121821</v>
       </c>
     </row>
     <row r="40">
@@ -2963,7 +2995,7 @@
       <c r="R40" t="inlineStr"/>
       <c r="S40" t="inlineStr"/>
       <c r="T40" t="n">
-        <v>1</v>
+        <v>0.1224486876578283</v>
       </c>
     </row>
     <row r="41">
@@ -3027,7 +3059,7 @@
         <v>0</v>
       </c>
       <c r="T41" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="42">
@@ -3079,7 +3111,7 @@
       <c r="R42" t="inlineStr"/>
       <c r="S42" t="inlineStr"/>
       <c r="T42" t="n">
-        <v>1</v>
+        <v>0.1224486876578283</v>
       </c>
     </row>
     <row r="43">
@@ -3143,7 +3175,7 @@
         <v>0</v>
       </c>
       <c r="T43" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="44">
@@ -3195,7 +3227,7 @@
       <c r="R44" t="inlineStr"/>
       <c r="S44" t="inlineStr"/>
       <c r="T44" t="n">
-        <v>1</v>
+        <v>0.1224486876578283</v>
       </c>
     </row>
     <row r="45">
@@ -3259,7 +3291,7 @@
         <v>0</v>
       </c>
       <c r="T45" t="n">
-        <v>1</v>
+        <v>0.2918963240121821</v>
       </c>
     </row>
     <row r="46">
@@ -3323,7 +3355,7 @@
         <v>0</v>
       </c>
       <c r="T46" t="n">
-        <v>1</v>
+        <v>0.2918963240121821</v>
       </c>
     </row>
     <row r="47">
@@ -3387,7 +3419,7 @@
         <v>0</v>
       </c>
       <c r="T47" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="48">
@@ -3451,7 +3483,7 @@
         <v>0</v>
       </c>
       <c r="T48" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="49">
@@ -3515,7 +3547,7 @@
         <v>0</v>
       </c>
       <c r="T49" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="50">
@@ -3579,7 +3611,7 @@
         <v>0</v>
       </c>
       <c r="T50" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="51">
@@ -3643,7 +3675,7 @@
         <v>0</v>
       </c>
       <c r="T51" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="52">
@@ -3707,7 +3739,7 @@
         <v>0</v>
       </c>
       <c r="T52" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="53">
@@ -3771,7 +3803,7 @@
         <v>0</v>
       </c>
       <c r="T53" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="54">
@@ -3835,7 +3867,7 @@
         <v>0</v>
       </c>
       <c r="T54" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="55">
@@ -3899,7 +3931,7 @@
         <v>0</v>
       </c>
       <c r="T55" t="n">
-        <v>1</v>
+        <v>0.2918963240121821</v>
       </c>
     </row>
     <row r="56">
@@ -3963,7 +3995,7 @@
         <v>0</v>
       </c>
       <c r="T56" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="57">
@@ -4027,7 +4059,7 @@
         <v>0</v>
       </c>
       <c r="T57" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="58">
@@ -4091,7 +4123,7 @@
         <v>0</v>
       </c>
       <c r="T58" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="59">
@@ -4155,7 +4187,7 @@
         <v>0</v>
       </c>
       <c r="T59" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="60">
@@ -4219,7 +4251,7 @@
         <v>0</v>
       </c>
       <c r="T60" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="61">
@@ -4283,7 +4315,7 @@
         <v>0</v>
       </c>
       <c r="T61" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="62">
@@ -4347,7 +4379,7 @@
         <v>0</v>
       </c>
       <c r="T62" t="n">
-        <v>1</v>
+        <v>0.2918963240121821</v>
       </c>
     </row>
     <row r="63">
@@ -4411,7 +4443,7 @@
         <v>0</v>
       </c>
       <c r="T63" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="64">
@@ -4475,7 +4507,7 @@
         <v>0</v>
       </c>
       <c r="T64" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="65">
@@ -4539,7 +4571,7 @@
         <v>0</v>
       </c>
       <c r="T65" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="66">
@@ -4603,7 +4635,7 @@
         <v>0</v>
       </c>
       <c r="T66" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="67">
@@ -4667,7 +4699,7 @@
         <v>0</v>
       </c>
       <c r="T67" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="68">
@@ -4731,7 +4763,7 @@
         <v>0</v>
       </c>
       <c r="T68" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="69">
@@ -4795,7 +4827,7 @@
         <v>0</v>
       </c>
       <c r="T69" t="n">
-        <v>1</v>
+        <v>0.2918963240121821</v>
       </c>
     </row>
     <row r="70">
@@ -4859,7 +4891,7 @@
         <v>0</v>
       </c>
       <c r="T70" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="71">
@@ -4923,7 +4955,7 @@
         <v>0</v>
       </c>
       <c r="T71" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="72">
@@ -4987,7 +5019,7 @@
         <v>0</v>
       </c>
       <c r="T72" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="73">
@@ -5051,7 +5083,7 @@
         <v>0</v>
       </c>
       <c r="T73" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="74">
@@ -5115,7 +5147,7 @@
         <v>0</v>
       </c>
       <c r="T74" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="75">
@@ -5179,7 +5211,7 @@
         <v>0</v>
       </c>
       <c r="T75" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="76">
@@ -5243,7 +5275,7 @@
         <v>0</v>
       </c>
       <c r="T76" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="77">
@@ -5307,7 +5339,7 @@
         <v>0</v>
       </c>
       <c r="T77" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="78">
@@ -5371,7 +5403,7 @@
         <v>0</v>
       </c>
       <c r="T78" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="79">
@@ -5435,7 +5467,7 @@
         <v>0</v>
       </c>
       <c r="T79" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="80">
@@ -5499,7 +5531,7 @@
         <v>0</v>
       </c>
       <c r="T80" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="81">
@@ -5563,7 +5595,7 @@
         <v>0</v>
       </c>
       <c r="T81" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="82">
@@ -5627,7 +5659,7 @@
         <v>0</v>
       </c>
       <c r="T82" t="n">
-        <v>1</v>
+        <v>0.2918963240121821</v>
       </c>
     </row>
     <row r="83">
@@ -5691,7 +5723,7 @@
         <v>0</v>
       </c>
       <c r="T83" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="84">
@@ -5755,7 +5787,7 @@
         <v>0</v>
       </c>
       <c r="T84" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="85">
@@ -5819,7 +5851,7 @@
         <v>0</v>
       </c>
       <c r="T85" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="86">
@@ -5883,7 +5915,7 @@
         <v>0</v>
       </c>
       <c r="T86" t="n">
-        <v>1</v>
+        <v>0.2918963240121821</v>
       </c>
     </row>
     <row r="87">
@@ -5947,7 +5979,7 @@
         <v>0</v>
       </c>
       <c r="T87" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="88">
@@ -6011,7 +6043,7 @@
         <v>0</v>
       </c>
       <c r="T88" t="n">
-        <v>1</v>
+        <v>0.2918963240121821</v>
       </c>
     </row>
     <row r="89">
@@ -6075,7 +6107,7 @@
         <v>0</v>
       </c>
       <c r="T89" t="n">
-        <v>1</v>
+        <v>0.2918963240121821</v>
       </c>
     </row>
     <row r="90">
@@ -6139,7 +6171,7 @@
         <v>0</v>
       </c>
       <c r="T90" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="91">
@@ -6203,7 +6235,7 @@
         <v>0</v>
       </c>
       <c r="T91" t="n">
-        <v>1</v>
+        <v>0.2918963240121821</v>
       </c>
     </row>
     <row r="92">
@@ -6267,7 +6299,7 @@
         <v>0</v>
       </c>
       <c r="T92" t="n">
-        <v>1</v>
+        <v>0.2918963240121821</v>
       </c>
     </row>
     <row r="93">
@@ -6331,7 +6363,7 @@
         <v>0</v>
       </c>
       <c r="T93" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="94">
@@ -6395,7 +6427,7 @@
         <v>0</v>
       </c>
       <c r="T94" t="n">
-        <v>1</v>
+        <v>0.2918963240121821</v>
       </c>
     </row>
     <row r="95">
@@ -6459,7 +6491,7 @@
         <v>0</v>
       </c>
       <c r="T95" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="96">
@@ -6523,7 +6555,7 @@
         <v>0</v>
       </c>
       <c r="T96" t="n">
-        <v>1</v>
+        <v>0.2918963240121821</v>
       </c>
     </row>
     <row r="97">
@@ -6587,7 +6619,7 @@
         <v>0</v>
       </c>
       <c r="T97" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="98">
@@ -6651,7 +6683,7 @@
         <v>0</v>
       </c>
       <c r="T98" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="99">
@@ -6715,7 +6747,7 @@
         <v>0</v>
       </c>
       <c r="T99" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="100">
@@ -6771,7 +6803,7 @@
       <c r="R100" t="inlineStr"/>
       <c r="S100" t="inlineStr"/>
       <c r="T100" t="n">
-        <v>1</v>
+        <v>0.01829346235012556</v>
       </c>
     </row>
     <row r="101">
@@ -6807,7 +6839,7 @@
       <c r="R101" t="inlineStr"/>
       <c r="S101" t="inlineStr"/>
       <c r="T101" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="102">
@@ -6869,7 +6901,7 @@
         <v>0</v>
       </c>
       <c r="T102" t="n">
-        <v>1</v>
+        <v>0.006622840730602443</v>
       </c>
     </row>
     <row r="103">
@@ -6933,7 +6965,7 @@
         <v>0</v>
       </c>
       <c r="T103" t="n">
-        <v>1</v>
+        <v>0.2918963240121821</v>
       </c>
     </row>
     <row r="104">
@@ -6997,7 +7029,7 @@
         <v>0</v>
       </c>
       <c r="T104" t="n">
-        <v>1</v>
+        <v>0.2918963240121821</v>
       </c>
     </row>
     <row r="105">
@@ -7053,7 +7085,7 @@
         <v>0</v>
       </c>
       <c r="T105" t="n">
-        <v>1</v>
+        <v>0.3789581051342651</v>
       </c>
     </row>
     <row r="106">
@@ -7109,7 +7141,7 @@
         <v>0</v>
       </c>
       <c r="T106" t="n">
-        <v>1</v>
+        <v>0.3789581051342651</v>
       </c>
     </row>
     <row r="107">
@@ -7165,7 +7197,7 @@
         <v>0</v>
       </c>
       <c r="T107" t="n">
-        <v>1</v>
+        <v>0.3789581051342651</v>
       </c>
     </row>
     <row r="108">
@@ -7221,7 +7253,7 @@
         <v>0</v>
       </c>
       <c r="T108" t="n">
-        <v>1</v>
+        <v>0.3789581051342651</v>
       </c>
     </row>
     <row r="109">
@@ -7277,7 +7309,7 @@
       <c r="R109" t="inlineStr"/>
       <c r="S109" t="inlineStr"/>
       <c r="T109" t="n">
-        <v>1</v>
+        <v>0.01829346235012556</v>
       </c>
     </row>
     <row r="110">
@@ -7313,7 +7345,7 @@
       <c r="R110" t="inlineStr"/>
       <c r="S110" t="inlineStr"/>
       <c r="T110" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="111">
@@ -7375,7 +7407,7 @@
         <v>0</v>
       </c>
       <c r="T111" t="n">
-        <v>1</v>
+        <v>0.006622840730602443</v>
       </c>
     </row>
     <row r="112">
@@ -7439,7 +7471,7 @@
         <v>0</v>
       </c>
       <c r="T112" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="113">
@@ -7503,7 +7535,7 @@
         <v>0</v>
       </c>
       <c r="T113" t="n">
-        <v>1</v>
+        <v>0.004720927622391452</v>
       </c>
     </row>
     <row r="114">
@@ -7559,7 +7591,7 @@
         <v>0</v>
       </c>
       <c r="T114" t="n">
-        <v>1</v>
+        <v>0.00612900416718784</v>
       </c>
     </row>
     <row r="115">
@@ -7615,7 +7647,7 @@
         <v>0</v>
       </c>
       <c r="T115" t="n">
-        <v>1</v>
+        <v>0.00612900416718784</v>
       </c>
     </row>
     <row r="116">
@@ -7671,7 +7703,7 @@
         <v>0</v>
       </c>
       <c r="T116" t="n">
-        <v>1</v>
+        <v>0.00612900416718784</v>
       </c>
     </row>
     <row r="117">
@@ -7727,7 +7759,7 @@
         <v>0</v>
       </c>
       <c r="T117" t="n">
-        <v>1</v>
+        <v>0.00612900416718784</v>
       </c>
     </row>
     <row r="118">
@@ -7785,7 +7817,7 @@
       </c>
       <c r="S118" t="inlineStr"/>
       <c r="T118" t="n">
-        <v>1</v>
+        <v>0.5292434375930891</v>
       </c>
     </row>
     <row r="119">
@@ -7843,7 +7875,7 @@
       </c>
       <c r="S119" t="inlineStr"/>
       <c r="T119" t="n">
-        <v>1</v>
+        <v>0.008559614349231567</v>
       </c>
     </row>
     <row r="120">
@@ -7901,7 +7933,7 @@
       </c>
       <c r="S120" t="inlineStr"/>
       <c r="T120" t="n">
-        <v>1</v>
+        <v>0.5292434375930891</v>
       </c>
     </row>
     <row r="121">
@@ -7959,7 +7991,7 @@
       </c>
       <c r="S121" t="inlineStr"/>
       <c r="T121" t="n">
-        <v>1</v>
+        <v>0.008559614349231567</v>
       </c>
     </row>
     <row r="122">
@@ -8017,7 +8049,7 @@
       </c>
       <c r="S122" t="inlineStr"/>
       <c r="T122" t="n">
-        <v>1</v>
+        <v>0.5292434375930891</v>
       </c>
     </row>
     <row r="123">
@@ -8075,7 +8107,7 @@
       </c>
       <c r="S123" t="inlineStr"/>
       <c r="T123" t="n">
-        <v>1</v>
+        <v>0.008559614349231567</v>
       </c>
     </row>
     <row r="124">
@@ -8133,7 +8165,7 @@
       </c>
       <c r="S124" t="inlineStr"/>
       <c r="T124" t="n">
-        <v>1</v>
+        <v>0.5292434375930891</v>
       </c>
     </row>
     <row r="125">
@@ -8191,7 +8223,7 @@
       </c>
       <c r="S125" t="inlineStr"/>
       <c r="T125" t="n">
-        <v>1</v>
+        <v>0.008559614349231567</v>
       </c>
     </row>
     <row r="126">
@@ -8249,7 +8281,7 @@
       </c>
       <c r="S126" t="inlineStr"/>
       <c r="T126" t="n">
-        <v>1</v>
+        <v>0.5292434375930891</v>
       </c>
     </row>
     <row r="127">
@@ -8307,7 +8339,7 @@
       </c>
       <c r="S127" t="inlineStr"/>
       <c r="T127" t="n">
-        <v>1</v>
+        <v>0.008559614349231567</v>
       </c>
     </row>
     <row r="128">
@@ -8365,7 +8397,7 @@
       </c>
       <c r="S128" t="inlineStr"/>
       <c r="T128" t="n">
-        <v>1</v>
+        <v>0.5292434375930891</v>
       </c>
     </row>
     <row r="129">
@@ -8423,7 +8455,7 @@
       </c>
       <c r="S129" t="inlineStr"/>
       <c r="T129" t="n">
-        <v>1</v>
+        <v>0.008559614349231567</v>
       </c>
     </row>
     <row r="130">
@@ -8481,7 +8513,7 @@
       </c>
       <c r="S130" t="inlineStr"/>
       <c r="T130" t="n">
-        <v>1</v>
+        <v>0.5292434375930891</v>
       </c>
     </row>
     <row r="131">
@@ -8539,7 +8571,7 @@
       </c>
       <c r="S131" t="inlineStr"/>
       <c r="T131" t="n">
-        <v>1</v>
+        <v>0.008559614349231567</v>
       </c>
     </row>
     <row r="132">
@@ -8597,7 +8629,7 @@
       </c>
       <c r="S132" t="inlineStr"/>
       <c r="T132" t="n">
-        <v>1</v>
+        <v>0.5292434375930891</v>
       </c>
     </row>
     <row r="133">
@@ -8655,7 +8687,7 @@
       </c>
       <c r="S133" t="inlineStr"/>
       <c r="T133" t="n">
-        <v>1</v>
+        <v>0.008559614349231567</v>
       </c>
     </row>
     <row r="134">
@@ -8713,7 +8745,7 @@
       </c>
       <c r="S134" t="inlineStr"/>
       <c r="T134" t="n">
-        <v>1</v>
+        <v>0.6081954192930815</v>
       </c>
     </row>
     <row r="135">
@@ -8771,7 +8803,7 @@
       </c>
       <c r="S135" t="inlineStr"/>
       <c r="T135" t="n">
-        <v>1</v>
+        <v>0.009836528652662409</v>
       </c>
     </row>
   </sheetData>

</xml_diff>